<commit_message>
NPCs, interaction to further prologue
</commit_message>
<xml_diff>
--- a/outline/Lost_Oracle_outline (version 1).xlsx
+++ b/outline/Lost_Oracle_outline (version 1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\msys64\home\patny\lost-oracle\outline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{4813006D-E36A-4F5F-8105-652D02CCB0F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{F8F15A84-B490-4820-BCEC-E0D98B89573A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{836BA816-2F37-4226-B892-498C904600FD}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="328">
   <si>
     <t>Town</t>
   </si>
@@ -997,6 +997,39 @@
   </si>
   <si>
     <t>(blank)</t>
+  </si>
+  <si>
+    <t>Fire Emblem The Blazing Blade - Requiem</t>
+  </si>
+  <si>
+    <t>Golden Sun - Lemuria</t>
+  </si>
+  <si>
+    <t>Deep Dark Galaxy</t>
+  </si>
+  <si>
+    <t>Dark Castle</t>
+  </si>
+  <si>
+    <t>Butter Canyon</t>
+  </si>
+  <si>
+    <t>Bowser's Lava Lake</t>
+  </si>
+  <si>
+    <t>Footlight Lane</t>
+  </si>
+  <si>
+    <t>Mount Magmeow</t>
+  </si>
+  <si>
+    <t>Mountain</t>
+  </si>
+  <si>
+    <t>Space Storm Galaxy</t>
+  </si>
+  <si>
+    <t>Night / Dungeon</t>
   </si>
 </sst>
 </file>
@@ -6754,116 +6787,179 @@
       </c>
     </row>
     <row r="122" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B122" t="s">
+        <v>34</v>
+      </c>
+      <c r="C122" t="s">
+        <v>317</v>
+      </c>
       <c r="H122" s="172" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="123" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B123" t="s">
+        <v>173</v>
+      </c>
+      <c r="C123" t="s">
+        <v>318</v>
+      </c>
       <c r="H123" s="30" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="124" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B124" t="s">
+        <v>173</v>
+      </c>
+      <c r="C124" t="s">
+        <v>319</v>
+      </c>
       <c r="H124" s="172" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="125" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B125" t="s">
+        <v>34</v>
+      </c>
+      <c r="C125" t="s">
+        <v>320</v>
+      </c>
       <c r="H125" s="30" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="126" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C126" t="s">
+        <v>321</v>
+      </c>
       <c r="H126" s="172" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="127" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B127" t="s">
+        <v>34</v>
+      </c>
+      <c r="C127" t="s">
+        <v>322</v>
+      </c>
       <c r="H127" s="30" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="128" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B128" t="s">
+        <v>173</v>
+      </c>
+      <c r="C128" t="s">
+        <v>323</v>
+      </c>
       <c r="H128" s="172" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="129" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B129" t="s">
+        <v>325</v>
+      </c>
+      <c r="C129" t="s">
+        <v>324</v>
+      </c>
       <c r="H129" s="172" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="130" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B130" t="s">
+        <v>173</v>
+      </c>
+      <c r="C130" t="s">
+        <v>240</v>
+      </c>
       <c r="H130" s="172" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="131" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B131" t="s">
+        <v>173</v>
+      </c>
+      <c r="C131" t="s">
+        <v>251</v>
+      </c>
       <c r="H131" s="30" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="132" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B132" t="s">
+        <v>327</v>
+      </c>
+      <c r="C132" t="s">
+        <v>326</v>
+      </c>
       <c r="H132" s="172" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="133" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H133" s="172" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="134" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H134" s="30" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="135" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H135" s="172" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="136" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H136" s="172" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="137" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H137" s="172" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="138" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H138" s="172" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="139" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H139" s="30" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="140" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H140" s="172" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="141" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H141" s="30" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="142" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H142" s="172" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="143" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H143" s="30" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="144" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H144" s="172" t="s">
         <v>266</v>
       </c>

</xml_diff>